<commit_message>
Figures in the company's style, and checked; KM table and figure in SAMPLE-01
- company standards gain figure_settings / figure_colors / figure_markers
  (built-in = tflspec's figure style, from the KM / waterfall / swimmer
  sample programs)
- saving writes programs/tfl/fig_setup.R; every figure program sources it
  and ends with tfl_check(plot), whose warnings the official run counts
- SAMPLE-01: ADTTE (time to first dermatologic event, derived from ADSL /
  ADAE), KM table T-14-2-2 and KM figure F-14-2-2 whose number at risk is
  the table's ARD (tfl_km_risk(), checked against the curve); F-14-2-1 uses
  the style helpers
- needs tflspec >= 0.0.6

Closes #5

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/listing_figure_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/listing_figure_spec.xlsx
@@ -623,7 +623,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -650,6 +650,18 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F-14-2-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ADTTE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sample study: its figures as user-code reports (#94)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/listing_figure_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/listing_figure_spec.xlsx
@@ -353,7 +353,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -385,6 +385,16 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>max_rows</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>blank_row</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>wrap</t>
         </is>
       </c>
     </row>
@@ -427,7 +437,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -453,6 +463,16 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>sep</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>align</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>collapse_repeats</t>
         </is>
       </c>
@@ -500,7 +520,7 @@
           <t>14</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -623,7 +643,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -637,6 +657,11 @@
           <t>datasets</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ard</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">

</xml_diff>

<commit_message>
The sample study and the table_data template, after the sample audit (#238)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/sample/SAMPLE-01/spec/listing_figure_spec.xlsx
+++ b/inst/sample/SAMPLE-01/spec/listing_figure_spec.xlsx
@@ -416,12 +416,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AESEV == "SEVERE"</t>
+          <t>AESEV == "SEVERE" &amp; TRTEMFL == "Y"</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TRT01A | USUBJID | ASTDT</t>
+          <t>TRT01AN | USUBJID | ASTDT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>